<commit_message>
Normal Deploy for ssecond test!
</commit_message>
<xml_diff>
--- a/PDD_voprosy_test1.xlsx
+++ b/PDD_voprosy_test1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Denis\Desktop\AplicationJavaFix\AutoSpace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C80E361-672B-4292-8CA3-E7FA82091E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA710269-1DF1-4F07-A0B6-B02790657D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="1808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="1814">
   <si>
     <t>test_number</t>
   </si>
@@ -5445,6 +5445,24 @@
   </si>
   <si>
     <t>Знак з ОДНІЄЮ діагональною смугою (R-308) забороняє саме парковку в цьому місці, але короткочасна зупинка (менше 2 хвилин, без виходу водія з машини) все ще дозволена. Знак із ДВОМА діагональними смугами (хрест, R-307) суворіший і забороняє і зупинку, і парковку без винятків.</t>
+  </si>
+  <si>
+    <t>question_key</t>
+  </si>
+  <si>
+    <t>question-31-a</t>
+  </si>
+  <si>
+    <t>question-32-b</t>
+  </si>
+  <si>
+    <t>question-33-c</t>
+  </si>
+  <si>
+    <t>question-47-a</t>
+  </si>
+  <si>
+    <t>question-47-b</t>
   </si>
 </sst>
 </file>
@@ -5667,7 +5685,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -5691,7 +5709,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -5701,7 +5719,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6114,7 +6132,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AG105"/>
+  <dimension ref="A1:AH105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6135,9 +6153,10 @@
     <col min="28" max="31" width="22" customWidth="1"/>
     <col min="32" max="32" width="35" customWidth="1"/>
     <col min="33" max="33" width="12" customWidth="1"/>
+    <col min="34" max="34" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -6237,8 +6256,11 @@
       <c r="AG1" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="AH1" s="4" t="s">
+        <v>1808</v>
+      </c>
     </row>
-    <row r="2" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -6338,8 +6360,11 @@
       <c r="AG2" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH2" s="10" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="3" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10">
         <v>1</v>
       </c>
@@ -6439,8 +6464,11 @@
       <c r="AG3" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH3" s="10" t="s">
+        <v>65</v>
+      </c>
     </row>
-    <row r="4" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10">
         <v>1</v>
       </c>
@@ -6540,8 +6568,11 @@
       <c r="AG4" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH4" s="10" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="5" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
         <v>1</v>
       </c>
@@ -6621,8 +6652,11 @@
       <c r="AG5" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="AH5" s="10" t="s">
+        <v>129</v>
+      </c>
     </row>
-    <row r="6" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10">
         <v>1</v>
       </c>
@@ -6722,8 +6756,11 @@
       <c r="AG6" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH6" s="10" t="s">
+        <v>150</v>
+      </c>
     </row>
-    <row r="7" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10">
         <v>1</v>
       </c>
@@ -6823,8 +6860,11 @@
       <c r="AG7" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH7" s="10" t="s">
+        <v>181</v>
+      </c>
     </row>
-    <row r="8" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10">
         <v>1</v>
       </c>
@@ -6924,8 +6964,11 @@
       <c r="AG8" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH8" s="10" t="s">
+        <v>212</v>
+      </c>
     </row>
-    <row r="9" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10">
         <v>1</v>
       </c>
@@ -7025,8 +7068,11 @@
       <c r="AG9" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH9" s="10" t="s">
+        <v>243</v>
+      </c>
     </row>
-    <row r="10" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10">
         <v>1</v>
       </c>
@@ -7126,8 +7172,11 @@
       <c r="AG10" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH10" s="10" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="11" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
         <v>1</v>
       </c>
@@ -7227,8 +7276,11 @@
       <c r="AG11" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH11" s="10" t="s">
+        <v>305</v>
+      </c>
     </row>
-    <row r="12" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10">
         <v>1</v>
       </c>
@@ -7328,8 +7380,11 @@
       <c r="AG12" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH12" s="10" t="s">
+        <v>336</v>
+      </c>
     </row>
-    <row r="13" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10">
         <v>1</v>
       </c>
@@ -7429,8 +7484,11 @@
       <c r="AG13" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH13" s="10" t="s">
+        <v>367</v>
+      </c>
     </row>
-    <row r="14" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
         <v>1</v>
       </c>
@@ -7530,8 +7588,11 @@
       <c r="AG14" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH14" s="10" t="s">
+        <v>398</v>
+      </c>
     </row>
-    <row r="15" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10">
         <v>1</v>
       </c>
@@ -7631,8 +7692,11 @@
       <c r="AG15" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH15" s="10" t="s">
+        <v>429</v>
+      </c>
     </row>
-    <row r="16" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10">
         <v>1</v>
       </c>
@@ -7732,8 +7796,11 @@
       <c r="AG16" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="AH16" s="10" t="s">
+        <v>460</v>
+      </c>
     </row>
-    <row r="17" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
         <v>1</v>
       </c>
@@ -7833,8 +7900,11 @@
       <c r="AG17" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH17" s="10" t="s">
+        <v>491</v>
+      </c>
     </row>
-    <row r="18" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10">
         <v>1</v>
       </c>
@@ -7934,8 +8004,11 @@
       <c r="AG18" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH18" s="10" t="s">
+        <v>522</v>
+      </c>
     </row>
-    <row r="19" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
         <v>1</v>
       </c>
@@ -8035,8 +8108,11 @@
       <c r="AG19" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="AH19" s="10" t="s">
+        <v>552</v>
+      </c>
     </row>
-    <row r="20" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
         <v>1</v>
       </c>
@@ -8136,8 +8212,11 @@
       <c r="AG20" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="AH20" s="10" t="s">
+        <v>583</v>
+      </c>
     </row>
-    <row r="21" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
         <v>1</v>
       </c>
@@ -8237,8 +8316,11 @@
       <c r="AG21" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH21" s="10" t="s">
+        <v>614</v>
+      </c>
     </row>
-    <row r="22" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
         <v>1</v>
       </c>
@@ -8338,8 +8420,11 @@
       <c r="AG22" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH22" s="10" t="s">
+        <v>645</v>
+      </c>
     </row>
-    <row r="23" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
         <v>1</v>
       </c>
@@ -8439,8 +8524,11 @@
       <c r="AG23" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH23" s="10" t="s">
+        <v>671</v>
+      </c>
     </row>
-    <row r="24" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
         <v>1</v>
       </c>
@@ -8540,8 +8628,11 @@
       <c r="AG24" s="10" t="s">
         <v>149</v>
       </c>
+      <c r="AH24" s="10" t="s">
+        <v>702</v>
+      </c>
     </row>
-    <row r="25" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
         <v>1</v>
       </c>
@@ -8641,8 +8732,11 @@
       <c r="AG25" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH25" s="10" t="s">
+        <v>733</v>
+      </c>
     </row>
-    <row r="26" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
         <v>1</v>
       </c>
@@ -8742,8 +8836,11 @@
       <c r="AG26" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH26" s="10" t="s">
+        <v>764</v>
+      </c>
     </row>
-    <row r="27" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10">
         <v>1</v>
       </c>
@@ -8843,8 +8940,11 @@
       <c r="AG27" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH27" s="10" t="s">
+        <v>795</v>
+      </c>
     </row>
-    <row r="28" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10">
         <v>1</v>
       </c>
@@ -8944,8 +9044,11 @@
       <c r="AG28" s="10" t="s">
         <v>128</v>
       </c>
+      <c r="AH28" s="10" t="s">
+        <v>821</v>
+      </c>
     </row>
-    <row r="29" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
         <v>1</v>
       </c>
@@ -9045,8 +9148,11 @@
       <c r="AG29" s="10" t="s">
         <v>64</v>
       </c>
+      <c r="AH29" s="10" t="s">
+        <v>852</v>
+      </c>
     </row>
-    <row r="30" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10">
         <v>1</v>
       </c>
@@ -9146,8 +9252,11 @@
       <c r="AG30" s="10" t="s">
         <v>96</v>
       </c>
+      <c r="AH30" s="10" t="s">
+        <v>883</v>
+      </c>
     </row>
-    <row r="31" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19">
         <v>1</v>
       </c>
@@ -9247,8 +9356,11 @@
       <c r="AG31" s="19" t="s">
         <v>96</v>
       </c>
+      <c r="AH31" s="10" t="s">
+        <v>909</v>
+      </c>
     </row>
-    <row r="32" spans="1:33" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:34" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16">
         <v>2</v>
       </c>
@@ -9348,8 +9460,11 @@
       <c r="AG32" s="16" t="s">
         <v>96</v>
       </c>
+      <c r="AH32" s="10" t="s">
+        <v>1809</v>
+      </c>
     </row>
-    <row r="33" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="16">
         <v>2</v>
       </c>
@@ -9449,8 +9564,11 @@
       <c r="AG33" s="26" t="s">
         <v>128</v>
       </c>
+      <c r="AH33" s="10" t="s">
+        <v>1810</v>
+      </c>
     </row>
-    <row r="34" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16">
         <v>2</v>
       </c>
@@ -9550,8 +9668,11 @@
       <c r="AG34" s="26" t="s">
         <v>96</v>
       </c>
+      <c r="AH34" s="10" t="s">
+        <v>1811</v>
+      </c>
     </row>
-    <row r="35" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="16">
         <v>2</v>
       </c>
@@ -9651,8 +9772,11 @@
       <c r="AG35" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH35" s="10" t="s">
+        <v>992</v>
+      </c>
     </row>
-    <row r="36" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="16">
         <v>2</v>
       </c>
@@ -9752,8 +9876,11 @@
       <c r="AG36" s="26" t="s">
         <v>96</v>
       </c>
+      <c r="AH36" s="10" t="s">
+        <v>993</v>
+      </c>
     </row>
-    <row r="37" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="16">
         <v>2</v>
       </c>
@@ -9853,8 +9980,11 @@
       <c r="AG37" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH37" s="10" t="s">
+        <v>994</v>
+      </c>
     </row>
-    <row r="38" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16">
         <v>2</v>
       </c>
@@ -9954,8 +10084,11 @@
       <c r="AG38" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH38" s="10" t="s">
+        <v>995</v>
+      </c>
     </row>
-    <row r="39" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="16">
         <v>2</v>
       </c>
@@ -10055,8 +10188,11 @@
       <c r="AG39" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH39" s="10" t="s">
+        <v>996</v>
+      </c>
     </row>
-    <row r="40" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16">
         <v>2</v>
       </c>
@@ -10156,8 +10292,11 @@
       <c r="AG40" s="26" t="s">
         <v>96</v>
       </c>
+      <c r="AH40" s="10" t="s">
+        <v>997</v>
+      </c>
     </row>
-    <row r="41" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="16">
         <v>2</v>
       </c>
@@ -10257,8 +10396,11 @@
       <c r="AG41" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH41" s="10" t="s">
+        <v>998</v>
+      </c>
     </row>
-    <row r="42" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="16">
         <v>2</v>
       </c>
@@ -10358,8 +10500,11 @@
       <c r="AG42" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH42" s="10" t="s">
+        <v>999</v>
+      </c>
     </row>
-    <row r="43" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="16">
         <v>2</v>
       </c>
@@ -10459,8 +10604,11 @@
       <c r="AG43" s="26" t="s">
         <v>96</v>
       </c>
+      <c r="AH43" s="10" t="s">
+        <v>1000</v>
+      </c>
     </row>
-    <row r="44" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="16">
         <v>2</v>
       </c>
@@ -10560,8 +10708,11 @@
       <c r="AG44" s="26" t="s">
         <v>96</v>
       </c>
+      <c r="AH44" s="10" t="s">
+        <v>1001</v>
+      </c>
     </row>
-    <row r="45" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16">
         <v>2</v>
       </c>
@@ -10661,8 +10812,11 @@
       <c r="AG45" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH45" s="10" t="s">
+        <v>1002</v>
+      </c>
     </row>
-    <row r="46" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16">
         <v>2</v>
       </c>
@@ -10762,8 +10916,11 @@
       <c r="AG46" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH46" s="10" t="s">
+        <v>1003</v>
+      </c>
     </row>
-    <row r="47" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="16">
         <v>2</v>
       </c>
@@ -10863,8 +11020,11 @@
       <c r="AG47" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH47" s="10" t="s">
+        <v>1004</v>
+      </c>
     </row>
-    <row r="48" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16">
         <v>2</v>
       </c>
@@ -10964,8 +11124,11 @@
       <c r="AG48" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH48" s="10" t="s">
+        <v>1812</v>
+      </c>
     </row>
-    <row r="49" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="16">
         <v>2</v>
       </c>
@@ -11065,8 +11228,11 @@
       <c r="AG49" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH49" s="10" t="s">
+        <v>1813</v>
+      </c>
     </row>
-    <row r="50" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16">
         <v>2</v>
       </c>
@@ -11166,8 +11332,11 @@
       <c r="AG50" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH50" s="10" t="s">
+        <v>1006</v>
+      </c>
     </row>
-    <row r="51" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16">
         <v>2</v>
       </c>
@@ -11267,8 +11436,11 @@
       <c r="AG51" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH51" s="10" t="s">
+        <v>1007</v>
+      </c>
     </row>
-    <row r="52" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16">
         <v>2</v>
       </c>
@@ -11368,8 +11540,11 @@
       <c r="AG52" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH52" s="10" t="s">
+        <v>1008</v>
+      </c>
     </row>
-    <row r="53" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16">
         <v>2</v>
       </c>
@@ -11469,8 +11644,11 @@
       <c r="AG53" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH53" s="10" t="s">
+        <v>1009</v>
+      </c>
     </row>
-    <row r="54" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16">
         <v>2</v>
       </c>
@@ -11570,8 +11748,11 @@
       <c r="AG54" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH54" s="10" t="s">
+        <v>1010</v>
+      </c>
     </row>
-    <row r="55" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16">
         <v>2</v>
       </c>
@@ -11671,8 +11852,11 @@
       <c r="AG55" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH55" s="10" t="s">
+        <v>1011</v>
+      </c>
     </row>
-    <row r="56" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16">
         <v>2</v>
       </c>
@@ -11772,8 +11956,11 @@
       <c r="AG56" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH56" s="10" t="s">
+        <v>1012</v>
+      </c>
     </row>
-    <row r="57" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="16">
         <v>2</v>
       </c>
@@ -11873,8 +12060,11 @@
       <c r="AG57" s="26" t="s">
         <v>64</v>
       </c>
+      <c r="AH57" s="10" t="s">
+        <v>1013</v>
+      </c>
     </row>
-    <row r="58" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="16">
         <v>2</v>
       </c>
@@ -11974,8 +12164,11 @@
       <c r="AG58" s="26" t="s">
         <v>149</v>
       </c>
+      <c r="AH58" s="10" t="s">
+        <v>1014</v>
+      </c>
     </row>
-    <row r="59" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="16">
         <v>2</v>
       </c>
@@ -12075,8 +12268,11 @@
       <c r="AG59" s="30" t="s">
         <v>149</v>
       </c>
+      <c r="AH59" s="10" t="s">
+        <v>1015</v>
+      </c>
     </row>
-    <row r="60" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="16">
         <v>2</v>
       </c>
@@ -12176,8 +12372,11 @@
       <c r="AG60" s="30" t="s">
         <v>149</v>
       </c>
+      <c r="AH60" s="10" t="s">
+        <v>1016</v>
+      </c>
     </row>
-    <row r="61" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="16">
         <v>2</v>
       </c>
@@ -12277,10 +12476,13 @@
       <c r="AG61" s="30" t="s">
         <v>64</v>
       </c>
+      <c r="AH61" s="10" t="s">
+        <v>1777</v>
+      </c>
     </row>
-    <row r="62" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:33" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:34" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="65" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="66" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12324,7 +12526,7 @@
     <row r="105" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" errorTitle="Неверное значение" error="Выберите A, B, C или D" sqref="AG2:AG1600" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"A,B,C,D"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Saving real stage of the test!
</commit_message>
<xml_diff>
--- a/PDD_voprosy_test1.xlsx
+++ b/PDD_voprosy_test1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Denis\Desktop\AplicationJavaFix\AutoSpace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA710269-1DF1-4F07-A0B6-B02790657D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4370A09F-2D84-4F63-9D72-F87ABF6EF339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5462,7 +5462,7 @@
     <t>question-47-a</t>
   </si>
   <si>
-    <t>question-47-b</t>
+    <t>question-48-b</t>
   </si>
 </sst>
 </file>

</xml_diff>